<commit_message>
Precisera Euler- och SSD-frågorna
- Euler: e är hans beteckning, π populariserade han (infördes av Jones)
- SSD: 'kommer åt data' i stället för 'kommer åt minnen'

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMyzzGMHCjJ5yybTsnetuR
</commit_message>
<xml_diff>
--- a/frågor_jeopardy_ny_omgång.xlsx
+++ b/frågor_jeopardy_ny_omgång.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Modern typ av hårddisk som kommer åt minnen snabbare än klassiska HDD</t>
+          <t>Modern typ av hårddisk som kommer åt data snabbare än klassiska HDD</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Historiens mest produktive matematiker som gav oss beteckningarna e och π samt arbetade vidare även som blind</t>
+          <t>Historiens mest produktive matematiker som gav oss beteckningen e, populariserade π och arbetade vidare även som blind</t>
         </is>
       </c>
     </row>

</xml_diff>